<commit_message>
SRS - Signal Process 수정 중간 커밋
</commit_message>
<xml_diff>
--- a/Document/RV201/RW-TF-FST-02-04 Attachment SRS List.xlsx
+++ b/Document/RV201/RW-TF-FST-02-04 Attachment SRS List.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Raywatt\Downloads\OneDrive_2025-02-24\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gordon\source\repos\RaywattOCT\Document\RV201\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2BB4419-100B-403A-B3FE-BBF24EFB4EC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{502599CE-AE9F-47B3-9BA2-EAA7C90F087A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{A2BBEDFD-6D56-46E5-86B3-01D2DB45E73E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A2BBEDFD-6D56-46E5-86B3-01D2DB45E73E}"/>
   </bookViews>
   <sheets>
     <sheet name="SRS" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="173">
   <si>
     <t>Data Communication Access Control</t>
     <phoneticPr fontId="4" type="noConversion"/>
@@ -251,53 +251,29 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>SRS-022</t>
-  </si>
-  <si>
     <t>Adjust Brightness</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>SRS-021</t>
-  </si>
-  <si>
     <t>Change Frame</t>
   </si>
   <si>
-    <t>SRS-020</t>
-  </si>
-  <si>
     <t>Change Degree</t>
   </si>
   <si>
-    <t>SRS-019</t>
-  </si>
-  <si>
     <t>Make L-View Image</t>
   </si>
   <si>
-    <t>SRS-018</t>
-  </si>
-  <si>
     <t>Save Raw Image</t>
   </si>
   <si>
-    <t>SRS-017</t>
-  </si>
-  <si>
     <t>Load Raw Image</t>
   </si>
   <si>
-    <t>SRS-016</t>
-  </si>
-  <si>
     <t>Convert OCT Signal to Image</t>
   </si>
   <si>
     <t>Signal Processing</t>
-  </si>
-  <si>
-    <t>SRS-015</t>
   </si>
   <si>
     <t>Acquire OCT Signal</t>
@@ -566,6 +542,36 @@
   </si>
   <si>
     <t>Only USB data communication is allowed, with wired and wireless communication restricted</t>
+  </si>
+  <si>
+    <t>Set Laser Module Setting</t>
+  </si>
+  <si>
+    <t>Set Sampling interval, Ascan, Bscan and etc..</t>
+  </si>
+  <si>
+    <t>Load System Calibraion File</t>
+  </si>
+  <si>
+    <t>Load Background, Map, Dispersion data from Specific Path</t>
+  </si>
+  <si>
+    <t>Get OCT Signal from Laser Module</t>
+  </si>
+  <si>
+    <t>Samples OCT signals from the laser module at a predefined interval</t>
+  </si>
+  <si>
+    <t>Remove Noise Signal from OCT Signal</t>
+  </si>
+  <si>
+    <t>Removing DC Noise and Speckle Noise from OCT Signal</t>
+  </si>
+  <si>
+    <t>Polarization Control</t>
+  </si>
+  <si>
+    <t>Find Maximum Peak Signal for finding Polarization-control Position</t>
   </si>
 </sst>
 </file>
@@ -617,7 +623,7 @@
       <charset val="129"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -627,6 +633,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -698,7 +710,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -721,13 +733,19 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -739,10 +757,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1080,7 +1110,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4F57D64-AE37-418E-9001-23E5658A302E}">
-  <dimension ref="A1:D52"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.5" style="2" bestFit="1" customWidth="1"/>
@@ -1092,672 +1122,707 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="D1" s="7" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>114</v>
+        <v>107</v>
+      </c>
+      <c r="B2" s="10" t="s">
+        <v>106</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="D2" s="14" t="s">
-        <v>120</v>
+        <v>105</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="B3" s="9"/>
+        <v>104</v>
+      </c>
+      <c r="B3" s="12"/>
       <c r="C3" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>121</v>
+        <v>103</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>110</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>109</v>
+        <v>102</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>101</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="D4" s="14" t="s">
-        <v>122</v>
+        <v>100</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="B5" s="10"/>
+        <v>99</v>
+      </c>
+      <c r="B5" s="11"/>
       <c r="C5" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="D5" s="14" t="s">
-        <v>123</v>
+        <v>98</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="B6" s="10"/>
+        <v>97</v>
+      </c>
+      <c r="B6" s="11"/>
       <c r="C6" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="D6" s="14" t="s">
-        <v>124</v>
+        <v>96</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="B7" s="9"/>
+        <v>95</v>
+      </c>
+      <c r="B7" s="12"/>
       <c r="C7" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="D7" s="14" t="s">
-        <v>125</v>
+        <v>94</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>100</v>
+        <v>93</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>92</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>126</v>
+        <v>91</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="B9" s="10"/>
+        <v>90</v>
+      </c>
+      <c r="B9" s="11"/>
       <c r="C9" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>127</v>
+        <v>89</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="B10" s="9"/>
+        <v>88</v>
+      </c>
+      <c r="B10" s="12"/>
       <c r="C10" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="D10" s="15" t="s">
-        <v>128</v>
+        <v>87</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>93</v>
+        <v>86</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>85</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="D11" s="15" t="s">
-        <v>129</v>
+        <v>84</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B12" s="10"/>
+        <v>83</v>
+      </c>
+      <c r="B12" s="11"/>
       <c r="C12" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="D12" s="15" t="s">
-        <v>130</v>
+        <v>82</v>
+      </c>
+      <c r="D12" s="9" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B13" s="10"/>
+        <v>81</v>
+      </c>
+      <c r="B13" s="11"/>
       <c r="C13" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>131</v>
+        <v>80</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B14" s="9"/>
+        <v>79</v>
+      </c>
+      <c r="B14" s="12"/>
       <c r="C14" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D14" s="15" t="s">
-        <v>132</v>
+        <v>78</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="D15" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="4"/>
+      <c r="B16" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="C16" s="19" t="s">
+        <v>163</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="4"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D17" s="20" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="4"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="21" t="s">
+        <v>167</v>
+      </c>
+      <c r="D18" s="20" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="4"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="21" t="s">
+        <v>169</v>
+      </c>
+      <c r="D19" s="20" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="4"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="E20" s="9"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="4"/>
+      <c r="B21" s="17"/>
+      <c r="C21" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="D21" s="20" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="4"/>
+      <c r="B22" s="17"/>
+      <c r="C22" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="4"/>
+      <c r="B23" s="17"/>
+      <c r="C23" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="4"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="4"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="4"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="D26" s="9" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="4"/>
+      <c r="B27" s="17"/>
+      <c r="C27" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D27" s="9" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="4"/>
+      <c r="B28" s="18"/>
+      <c r="C28" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="D28" s="9" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="D16" s="15" t="s">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B29" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D29" s="9" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B17" s="10"/>
-      <c r="C17" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="D17" s="15" t="s">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="B30" s="17"/>
+      <c r="C30" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D30" s="9" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B18" s="10"/>
-      <c r="C18" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="D18" s="15" t="s">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B31" s="17"/>
+      <c r="C31" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D31" s="9" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B19" s="10"/>
-      <c r="C19" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D19" s="15" t="s">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="B32" s="17"/>
+      <c r="C32" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D32" s="9" t="s">
         <v>137</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="B21" s="10"/>
-      <c r="C21" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="D21" s="15" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A22" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B22" s="10"/>
-      <c r="C22" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="D22" s="15" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A23" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B23" s="9"/>
-      <c r="C23" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="D23" s="15" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A25" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B25" s="10"/>
-      <c r="C25" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="D25" s="15" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="B26" s="10"/>
-      <c r="C26" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="D26" s="15" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="B27" s="10"/>
-      <c r="C27" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D27" s="15" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A28" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="B28" s="9"/>
-      <c r="C28" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D28" s="15" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A29" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="B29" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="D29" s="15" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B30" s="10"/>
-      <c r="C30" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="D30" s="15" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A31" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B31" s="10"/>
-      <c r="C31" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="D31" s="15" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="B32" s="10"/>
-      <c r="C32" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D32" s="15" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B33" s="9"/>
+        <v>56</v>
+      </c>
+      <c r="B33" s="18"/>
       <c r="C33" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="D33" s="15" t="s">
-        <v>151</v>
+        <v>55</v>
+      </c>
+      <c r="D33" s="9" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="B34" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="D34" s="14" t="s">
-        <v>152</v>
+        <v>54</v>
+      </c>
+      <c r="B34" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="D34" s="9" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B35" s="10"/>
-      <c r="C35" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="D35" s="14" t="s">
-        <v>153</v>
+        <v>51</v>
+      </c>
+      <c r="B35" s="11"/>
+      <c r="C35" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D35" s="9" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B36" s="10"/>
-      <c r="C36" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="D36" s="14" t="s">
-        <v>154</v>
+        <v>49</v>
+      </c>
+      <c r="B36" s="11"/>
+      <c r="C36" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>141</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B37" s="10"/>
-      <c r="C37" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="D37" s="14" t="s">
-        <v>155</v>
+        <v>47</v>
+      </c>
+      <c r="B37" s="11"/>
+      <c r="C37" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B38" s="9"/>
-      <c r="C38" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="D38" s="14" t="s">
-        <v>156</v>
+        <v>45</v>
+      </c>
+      <c r="B38" s="12"/>
+      <c r="C38" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B39" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C39" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D39" s="15" t="s">
-        <v>157</v>
+        <v>43</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B40" s="10"/>
-      <c r="C40" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D40" s="15" t="s">
-        <v>158</v>
+        <v>40</v>
+      </c>
+      <c r="B40" s="11"/>
+      <c r="C40" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B41" s="10"/>
-      <c r="C41" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="D41" s="15" t="s">
-        <v>159</v>
+        <v>38</v>
+      </c>
+      <c r="B41" s="11"/>
+      <c r="C41" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D41" s="8" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B42" s="9"/>
-      <c r="C42" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="D42" s="15" t="s">
-        <v>160</v>
+        <v>36</v>
+      </c>
+      <c r="B42" s="11"/>
+      <c r="C42" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D42" s="8" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D43" s="15" t="s">
-        <v>161</v>
+        <v>34</v>
+      </c>
+      <c r="B43" s="12"/>
+      <c r="C43" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D43" s="8" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B44" s="9"/>
+        <v>32</v>
+      </c>
+      <c r="B44" s="10" t="s">
+        <v>31</v>
+      </c>
       <c r="C44" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D44" s="15" t="s">
-        <v>162</v>
+        <v>30</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B45" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="D45" s="14" t="s">
-        <v>163</v>
+        <v>29</v>
+      </c>
+      <c r="B45" s="11"/>
+      <c r="C45" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B46" s="10"/>
-      <c r="C46" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D46" s="14" t="s">
-        <v>164</v>
+        <v>27</v>
+      </c>
+      <c r="B46" s="11"/>
+      <c r="C46" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D46" s="9" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B47" s="9"/>
+        <v>25</v>
+      </c>
+      <c r="B47" s="12"/>
       <c r="C47" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D47" s="15" t="s">
-        <v>165</v>
+        <v>24</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="B48" s="4" t="s">
-        <v>10</v>
+        <v>23</v>
+      </c>
+      <c r="B48" s="10" t="s">
+        <v>22</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D48" s="15" t="s">
-        <v>166</v>
+        <v>21</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B49" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>167</v>
+        <v>20</v>
+      </c>
+      <c r="B49" s="12"/>
+      <c r="C49" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="B50" s="12"/>
-      <c r="C50" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D50" s="3" t="s">
-        <v>168</v>
+        <v>18</v>
+      </c>
+      <c r="B50" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D50" s="8" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B51" s="12"/>
-      <c r="C51" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D51" s="3" t="s">
-        <v>169</v>
+        <v>15</v>
+      </c>
+      <c r="B51" s="11"/>
+      <c r="C51" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D51" s="8" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B52" s="12"/>
+      <c r="C52" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A53" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D53" s="9" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B54" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B55" s="14"/>
+      <c r="C55" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="D55" s="3" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A56" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B56" s="14"/>
+      <c r="C56" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A57" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B52" s="13"/>
-      <c r="C52" s="3" t="s">
+      <c r="B57" s="15"/>
+      <c r="C57" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="D52" s="3" t="s">
-        <v>170</v>
+      <c r="D57" s="3" t="s">
+        <v>162</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="B45:B47"/>
-    <mergeCell ref="B49:B52"/>
-    <mergeCell ref="B24:B28"/>
-    <mergeCell ref="B29:B33"/>
-    <mergeCell ref="B34:B38"/>
-    <mergeCell ref="B39:B42"/>
-    <mergeCell ref="B43:B44"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="B4:B7"/>
     <mergeCell ref="B8:B10"/>
     <mergeCell ref="B11:B14"/>
-    <mergeCell ref="B16:B23"/>
+    <mergeCell ref="B16:B28"/>
+    <mergeCell ref="B50:B52"/>
+    <mergeCell ref="B54:B57"/>
+    <mergeCell ref="B29:B33"/>
+    <mergeCell ref="B34:B38"/>
+    <mergeCell ref="B39:B43"/>
+    <mergeCell ref="B44:B47"/>
+    <mergeCell ref="B48:B49"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1765,6 +1830,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="문서" ma:contentTypeID="0x01010055643D1FCDD1AF449E52FCC5650E658B" ma:contentTypeVersion="14" ma:contentTypeDescription="새 문서를 만듭니다." ma:contentTypeScope="" ma:versionID="647bdb025269980e27106cc2d7c93b4b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e9585e3e-8dde-4558-9020-300460070f66" xmlns:ns3="fdbd0ee6-c1ce-4682-bf4d-b990274ef7f9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d9d8955b532099d955db877a9cb0cef3" ns2:_="" ns3:_="">
     <xsd:import namespace="e9585e3e-8dde-4558-9020-300460070f66"/>
@@ -1977,15 +2051,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1998,13 +2063,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B3FA20A-BD9F-4422-9B89-7C75BEBC07A8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86FB0506-72B3-4F03-B05C-01BAB7410BED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86FB0506-72B3-4F03-B05C-01BAB7410BED}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B3FA20A-BD9F-4422-9B89-7C75BEBC07A8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e9585e3e-8dde-4558-9020-300460070f66"/>
+    <ds:schemaRef ds:uri="fdbd0ee6-c1ce-4682-bf4d-b990274ef7f9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DDE60D44-15A8-45C5-B02F-5E97D9FCFB03}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DDE60D44-15A8-45C5-B02F-5E97D9FCFB03}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="e9585e3e-8dde-4558-9020-300460070f66"/>
+    <ds:schemaRef ds:uri="fdbd0ee6-c1ce-4682-bf4d-b990274ef7f9"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
SRS 취합(UI, Angio 추가)
</commit_message>
<xml_diff>
--- a/Document/RV201/RW-TF-FST-02-04 Attachment SRS List.xlsx
+++ b/Document/RV201/RW-TF-FST-02-04 Attachment SRS List.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gordon\source\repos\RaywattOCT\Document\RV201\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93D6CBC1-3BF8-432F-A4D2-4BA02D6110AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F496664-B009-4FF9-9EA1-2BEB682C8DCD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A2BBEDFD-6D56-46E5-86B3-01D2DB45E73E}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="207">
   <si>
     <t>Convert OCT Image to DICOM Format</t>
   </si>
@@ -45,33 +45,6 @@
   </si>
   <si>
     <t>Image Processing</t>
-  </si>
-  <si>
-    <t>Send Angio Image</t>
-  </si>
-  <si>
-    <t>Acquire Angio Image</t>
-  </si>
-  <si>
-    <t>Angio Server</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>Save Angio Raw Image</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>Load Angio Raw Image</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
-    <t>Get Angio Image</t>
-  </si>
-  <si>
-    <t>Control Angio Server</t>
-  </si>
-  <si>
-    <t>Angio Client</t>
   </si>
   <si>
     <t>Make an Annotation</t>
@@ -166,13 +139,6 @@
     <t>DB Processing</t>
   </si>
   <si>
-    <t>Dialog UI</t>
-  </si>
-  <si>
-    <t>Page UI</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>UI Display</t>
   </si>
   <si>
@@ -191,12 +157,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>Page display</t>
-  </si>
-  <si>
-    <t>Dialog display</t>
-  </si>
-  <si>
     <t>Data input into Database</t>
   </si>
   <si>
@@ -222,24 +182,6 @@
   </si>
   <si>
     <t>Annotation creation</t>
-  </si>
-  <si>
-    <t>Angio Server process control</t>
-  </si>
-  <si>
-    <t>Receiving Angio Image from Angio Server</t>
-  </si>
-  <si>
-    <t>Loading Angio Raw Image file</t>
-  </si>
-  <si>
-    <t>Saving Angio Raw Image file</t>
-  </si>
-  <si>
-    <t>Acquiring Angio Image from Angio equipment</t>
-  </si>
-  <si>
-    <t>Transmitting acquired Angio Image to Angio Client</t>
   </si>
   <si>
     <t>Converting Export Image to DICOM format</t>
@@ -663,6 +605,100 @@
       <t>configuration changes, data retrieval, data creation, data modification, and data deletion events, including the timestamp for each logged event.</t>
     </r>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>The UI shall provide an admin screen that displays institution information and a user list, and supports user management functions..</t>
+  </si>
+  <si>
+    <t>Admin Login</t>
+  </si>
+  <si>
+    <t>The UI shall authenticate administrators using an ID and password before access is granted.</t>
+  </si>
+  <si>
+    <t>File I/O</t>
+  </si>
+  <si>
+    <t>The UI shall provide an import and export interface for handling patient and case data.</t>
+  </si>
+  <si>
+    <t>Home</t>
+  </si>
+  <si>
+    <t>The UI shall provide a home screen showing the patient list, device status icons, and navigation menus.</t>
+  </si>
+  <si>
+    <t>Loading</t>
+  </si>
+  <si>
+    <t>The UI shall display a progress indicator during system initialization after login.</t>
+  </si>
+  <si>
+    <t>Patient</t>
+  </si>
+  <si>
+    <t>The UI shall provide patient selection and patient information management functions.</t>
+  </si>
+  <si>
+    <t>Physician</t>
+  </si>
+  <si>
+    <t>The UI shall provide physician search and management functions.</t>
+  </si>
+  <si>
+    <t>Recording</t>
+  </si>
+  <si>
+    <t>The UI shall provide interfaces for configuring pullback options and starting OCT/Angio recording.</t>
+  </si>
+  <si>
+    <t>Review</t>
+  </si>
+  <si>
+    <t>The UI shall provide review interfaces for 2D/3D image viewing and measurement tools.</t>
+  </si>
+  <si>
+    <t>Settings</t>
+  </si>
+  <si>
+    <t>The UI shall provide system settings including storage, log export, and DICOM configuration.</t>
+  </si>
+  <si>
+    <t>System</t>
+  </si>
+  <si>
+    <t>The UI shall provide logout and shutdown dialogs for system control.</t>
+  </si>
+  <si>
+    <t>Terms</t>
+  </si>
+  <si>
+    <t>The UI shall display the Terms and Conditions and allow users to accept or decline.</t>
+  </si>
+  <si>
+    <t>User Login</t>
+  </si>
+  <si>
+    <t>The UI shall authenticate users using an ID and password before accessing user functions.</t>
+  </si>
+  <si>
+    <t>Angio</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Client</t>
+  </si>
+  <si>
+    <t>The system shall the system shall allow the Angio Client to manage Angio Server operations, including establishing, maintaining, and re-establishing the server connection as required.</t>
+  </si>
+  <si>
+    <t>Server</t>
+  </si>
+  <si>
+    <t>The system shall the system shall acquire Angio Image data directly from the connected Angio equipment in real time, ensuring accurate capture of imaging information.</t>
   </si>
 </sst>
 </file>
@@ -859,47 +895,20 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -910,6 +919,33 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1246,954 +1282,1021 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4F57D64-AE37-418E-9001-23E5658A302E}">
-  <dimension ref="A1:D89"/>
+  <dimension ref="A1:D96"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.5" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="20.25" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="33.875" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="127.25" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="155.125" style="2" bestFit="1" customWidth="1"/>
     <col min="5" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
-        <v>44</v>
+        <v>34</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>47</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
-      <c r="B2" s="10" t="s">
-        <v>43</v>
+      <c r="B2" s="22" t="s">
+        <v>33</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>42</v>
+        <v>176</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>48</v>
+        <v>177</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
-      <c r="B3" s="12"/>
+      <c r="B3" s="24"/>
       <c r="C3" s="5" t="s">
-        <v>41</v>
+        <v>178</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>49</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="3"/>
-      <c r="B4" s="10" t="s">
-        <v>40</v>
-      </c>
+      <c r="B4" s="24"/>
       <c r="C4" s="5" t="s">
-        <v>39</v>
+        <v>180</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>50</v>
+        <v>181</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="3"/>
-      <c r="B5" s="11"/>
+      <c r="B5" s="24"/>
       <c r="C5" s="5" t="s">
-        <v>38</v>
+        <v>182</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>51</v>
+        <v>183</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
-      <c r="B6" s="11"/>
+      <c r="B6" s="24"/>
       <c r="C6" s="5" t="s">
-        <v>37</v>
+        <v>184</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>52</v>
+        <v>185</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="3"/>
-      <c r="B7" s="12"/>
+      <c r="B7" s="24"/>
       <c r="C7" s="5" t="s">
-        <v>36</v>
+        <v>186</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>53</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
-      <c r="B8" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" s="24" t="s">
-        <v>167</v>
-      </c>
-      <c r="D8" s="24" t="s">
-        <v>168</v>
+      <c r="B8" s="24"/>
+      <c r="C8" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" s="3"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="24" t="s">
-        <v>169</v>
-      </c>
-      <c r="D9" s="24" t="s">
-        <v>170</v>
+      <c r="B9" s="24"/>
+      <c r="C9" s="5" t="s">
+        <v>190</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" s="3"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="24" t="s">
-        <v>171</v>
-      </c>
-      <c r="D10" s="24" t="s">
-        <v>172</v>
+      <c r="B10" s="24"/>
+      <c r="C10" s="5" t="s">
+        <v>192</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" s="3"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="24" t="s">
-        <v>173</v>
-      </c>
-      <c r="D11" s="24" t="s">
-        <v>174</v>
+      <c r="B11" s="24"/>
+      <c r="C11" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" s="3"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="24" t="s">
-        <v>175</v>
-      </c>
-      <c r="D12" s="24" t="s">
-        <v>176</v>
+      <c r="B12" s="24"/>
+      <c r="C12" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>197</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" s="3"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="24" t="s">
-        <v>177</v>
-      </c>
-      <c r="D13" s="24" t="s">
-        <v>178</v>
+      <c r="B13" s="24"/>
+      <c r="C13" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>199</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14" s="3"/>
-      <c r="B14" s="11"/>
-      <c r="C14" s="24" t="s">
-        <v>179</v>
-      </c>
-      <c r="D14" s="24" t="s">
-        <v>180</v>
+      <c r="B14" s="23"/>
+      <c r="C14" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" s="3"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="24" t="s">
-        <v>181</v>
-      </c>
-      <c r="D15" s="24" t="s">
-        <v>182</v>
+      <c r="B15" s="22" t="s">
+        <v>32</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" s="3"/>
-      <c r="B16" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C16" s="25" t="s">
-        <v>183</v>
-      </c>
-      <c r="D16" s="24" t="s">
-        <v>184</v>
+      <c r="B16" s="24"/>
+      <c r="C16" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="3"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="25" t="s">
-        <v>185</v>
-      </c>
-      <c r="D17" s="24" t="s">
-        <v>186</v>
+      <c r="B17" s="24"/>
+      <c r="C17" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="3"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="25" t="s">
-        <v>33</v>
-      </c>
-      <c r="D18" s="24" t="s">
-        <v>187</v>
+      <c r="B18" s="23"/>
+      <c r="C18" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="3"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="25" t="s">
-        <v>32</v>
-      </c>
-      <c r="D19" s="24" t="s">
-        <v>188</v>
+      <c r="B19" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="3"/>
-      <c r="B20" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="C20" s="24" t="s">
-        <v>189</v>
-      </c>
-      <c r="D20" s="24" t="s">
-        <v>190</v>
+      <c r="B20" s="24"/>
+      <c r="C20" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>152</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="3"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="24" t="s">
-        <v>191</v>
-      </c>
-      <c r="D21" s="24" t="s">
-        <v>192</v>
+      <c r="B21" s="24"/>
+      <c r="C21" s="15" t="s">
+        <v>153</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>154</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="3"/>
-      <c r="B22" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="C22" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="D22" s="24" t="s">
-        <v>75</v>
+      <c r="B22" s="24"/>
+      <c r="C22" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="3"/>
-      <c r="B23" s="17"/>
-      <c r="C23" s="24" t="s">
-        <v>76</v>
-      </c>
-      <c r="D23" s="24" t="s">
-        <v>77</v>
+      <c r="B23" s="24"/>
+      <c r="C23" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="3"/>
-      <c r="B24" s="17"/>
-      <c r="C24" s="24" t="s">
-        <v>67</v>
-      </c>
-      <c r="D24" s="24" t="s">
-        <v>78</v>
+      <c r="B24" s="24"/>
+      <c r="C24" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="3"/>
-      <c r="B25" s="17"/>
-      <c r="C25" s="24" t="s">
-        <v>68</v>
-      </c>
-      <c r="D25" s="24" t="s">
-        <v>79</v>
+      <c r="B25" s="24"/>
+      <c r="C25" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="3"/>
-      <c r="B26" s="17"/>
-      <c r="C26" s="24" t="s">
-        <v>29</v>
-      </c>
-      <c r="D26" s="24" t="s">
-        <v>80</v>
+      <c r="B26" s="23"/>
+      <c r="C26" s="15" t="s">
+        <v>163</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="3"/>
-      <c r="B27" s="17"/>
-      <c r="C27" s="24" t="s">
-        <v>81</v>
-      </c>
-      <c r="D27" s="24" t="s">
-        <v>82</v>
+      <c r="B27" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27" s="16" t="s">
+        <v>165</v>
+      </c>
+      <c r="D27" s="15" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="3"/>
-      <c r="B28" s="17"/>
-      <c r="C28" s="24" t="s">
-        <v>83</v>
-      </c>
-      <c r="D28" s="24" t="s">
-        <v>84</v>
+      <c r="B28" s="24"/>
+      <c r="C28" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="D28" s="15" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="3"/>
-      <c r="B29" s="17"/>
-      <c r="C29" s="24" t="s">
-        <v>28</v>
-      </c>
-      <c r="D29" s="24" t="s">
-        <v>85</v>
+      <c r="B29" s="24"/>
+      <c r="C29" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="3"/>
-      <c r="B30" s="17"/>
-      <c r="C30" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="D30" s="24" t="s">
-        <v>86</v>
+      <c r="B30" s="23"/>
+      <c r="C30" s="16" t="s">
+        <v>24</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="3"/>
-      <c r="B31" s="17"/>
-      <c r="C31" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="D31" s="24" t="s">
-        <v>87</v>
+      <c r="B31" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="3"/>
-      <c r="B32" s="17"/>
-      <c r="C32" s="24" t="s">
-        <v>25</v>
-      </c>
-      <c r="D32" s="24" t="s">
-        <v>88</v>
+      <c r="B32" s="23"/>
+      <c r="C32" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="3"/>
-      <c r="B33" s="17"/>
-      <c r="C33" s="24" t="s">
-        <v>24</v>
-      </c>
-      <c r="D33" s="24" t="s">
-        <v>89</v>
+      <c r="B33" s="25" t="s">
+        <v>22</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="3"/>
-      <c r="B34" s="17"/>
-      <c r="C34" s="24" t="s">
-        <v>90</v>
-      </c>
-      <c r="D34" s="24" t="s">
-        <v>91</v>
+      <c r="B34" s="26"/>
+      <c r="C34" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="3"/>
-      <c r="B35" s="19"/>
-      <c r="C35" s="24" t="s">
-        <v>92</v>
-      </c>
-      <c r="D35" s="24" t="s">
-        <v>93</v>
+      <c r="B35" s="26"/>
+      <c r="C35" s="15" t="s">
+        <v>49</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="3"/>
-      <c r="B36" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="C36" s="24" t="s">
-        <v>94</v>
-      </c>
-      <c r="D36" s="24" t="s">
-        <v>95</v>
+      <c r="B36" s="26"/>
+      <c r="C36" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="3"/>
-      <c r="B37" s="17"/>
-      <c r="C37" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="D37" s="24" t="s">
-        <v>96</v>
+      <c r="B37" s="26"/>
+      <c r="C37" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="3"/>
-      <c r="B38" s="17"/>
-      <c r="C38" s="24" t="s">
-        <v>21</v>
-      </c>
-      <c r="D38" s="24" t="s">
-        <v>97</v>
+      <c r="B38" s="26"/>
+      <c r="C38" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="3"/>
-      <c r="B39" s="17"/>
-      <c r="C39" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="D39" s="24" t="s">
-        <v>98</v>
+      <c r="B39" s="26"/>
+      <c r="C39" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="D39" s="15" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="3"/>
-      <c r="B40" s="17"/>
-      <c r="C40" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="D40" s="24" t="s">
-        <v>99</v>
+      <c r="B40" s="26"/>
+      <c r="C40" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="D40" s="15" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="3"/>
-      <c r="B41" s="17"/>
-      <c r="C41" s="24" t="s">
-        <v>18</v>
-      </c>
-      <c r="D41" s="24" t="s">
-        <v>100</v>
+      <c r="B41" s="26"/>
+      <c r="C41" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D41" s="15" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="3"/>
-      <c r="B42" s="19"/>
-      <c r="C42" s="24" t="s">
-        <v>101</v>
-      </c>
-      <c r="D42" s="24" t="s">
-        <v>102</v>
+      <c r="B42" s="26"/>
+      <c r="C42" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D42" s="15" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="3"/>
-      <c r="B43" s="10" t="s">
+      <c r="B43" s="26"/>
+      <c r="C43" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="C43" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="D43" s="8" t="s">
-        <v>146</v>
+      <c r="D43" s="15" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="3"/>
-      <c r="B44" s="11"/>
-      <c r="C44" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="D44" s="8" t="s">
-        <v>148</v>
+      <c r="B44" s="26"/>
+      <c r="C44" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="D44" s="15" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="3"/>
-      <c r="B45" s="11"/>
-      <c r="C45" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="D45" s="8" t="s">
-        <v>150</v>
+      <c r="B45" s="26"/>
+      <c r="C45" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="D45" s="15" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="3"/>
-      <c r="B46" s="11"/>
-      <c r="C46" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="D46" s="8" t="s">
-        <v>152</v>
+      <c r="B46" s="27"/>
+      <c r="C46" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="D46" s="15" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="3"/>
-      <c r="B47" s="11"/>
-      <c r="C47" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="D47" s="8" t="s">
-        <v>154</v>
+      <c r="B47" s="25" t="s">
+        <v>15</v>
+      </c>
+      <c r="C47" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="D47" s="15" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="3"/>
-      <c r="B48" s="11"/>
-      <c r="C48" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="D48" s="8" t="s">
-        <v>156</v>
+      <c r="B48" s="26"/>
+      <c r="C48" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D48" s="15" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="3"/>
-      <c r="B49" s="11"/>
-      <c r="C49" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="D49" s="8" t="s">
-        <v>158</v>
+      <c r="B49" s="26"/>
+      <c r="C49" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D49" s="15" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="3"/>
-      <c r="B50" s="11"/>
-      <c r="C50" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="D50" s="8" t="s">
-        <v>160</v>
+      <c r="B50" s="26"/>
+      <c r="C50" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D50" s="15" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="3"/>
-      <c r="B51" s="11"/>
-      <c r="C51" s="4" t="s">
-        <v>161</v>
-      </c>
-      <c r="D51" s="8" t="s">
-        <v>162</v>
+      <c r="B51" s="26"/>
+      <c r="C51" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D51" s="15" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="3"/>
-      <c r="B52" s="11"/>
-      <c r="C52" s="4" t="s">
-        <v>163</v>
-      </c>
-      <c r="D52" s="8" t="s">
-        <v>164</v>
+      <c r="B52" s="26"/>
+      <c r="C52" s="15" t="s">
+        <v>10</v>
+      </c>
+      <c r="D52" s="15" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="3"/>
-      <c r="B53" s="12"/>
-      <c r="C53" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="D53" s="8" t="s">
-        <v>166</v>
+      <c r="B53" s="27"/>
+      <c r="C53" s="15" t="s">
+        <v>83</v>
+      </c>
+      <c r="D53" s="15" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="3"/>
-      <c r="B54" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C54" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D54" s="7" t="s">
-        <v>54</v>
+      <c r="B54" s="22" t="s">
+        <v>9</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="D54" s="8" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" s="3"/>
-      <c r="B55" s="11"/>
-      <c r="C55" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D55" s="7" t="s">
-        <v>55</v>
+      <c r="B55" s="24"/>
+      <c r="C55" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="D55" s="8" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" s="3"/>
-      <c r="B56" s="11"/>
-      <c r="C56" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="D56" s="7" t="s">
-        <v>56</v>
+      <c r="B56" s="24"/>
+      <c r="C56" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="D56" s="8" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" s="3"/>
-      <c r="B57" s="11"/>
-      <c r="C57" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D57" s="7" t="s">
-        <v>57</v>
+      <c r="B57" s="24"/>
+      <c r="C57" s="4" t="s">
+        <v>133</v>
+      </c>
+      <c r="D57" s="8" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" s="3"/>
-      <c r="B58" s="11"/>
-      <c r="C58" s="26" t="s">
-        <v>69</v>
-      </c>
-      <c r="D58" s="26" t="s">
-        <v>70</v>
+      <c r="B58" s="24"/>
+      <c r="C58" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="D58" s="8" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" s="3"/>
-      <c r="B59" s="12"/>
-      <c r="C59" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="D59" s="9" t="s">
-        <v>58</v>
+      <c r="B59" s="24"/>
+      <c r="C59" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="D59" s="8" t="s">
+        <v>138</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" s="3"/>
-      <c r="B60" s="10" t="s">
-        <v>10</v>
-      </c>
+      <c r="B60" s="24"/>
       <c r="C60" s="4" t="s">
-        <v>9</v>
+        <v>139</v>
       </c>
       <c r="D60" s="8" t="s">
-        <v>59</v>
+        <v>140</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" s="3"/>
-      <c r="B61" s="11"/>
+      <c r="B61" s="24"/>
       <c r="C61" s="4" t="s">
-        <v>8</v>
+        <v>141</v>
       </c>
       <c r="D61" s="8" t="s">
-        <v>60</v>
+        <v>142</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" s="3"/>
-      <c r="B62" s="11"/>
+      <c r="B62" s="24"/>
       <c r="C62" s="4" t="s">
-        <v>7</v>
+        <v>143</v>
       </c>
       <c r="D62" s="8" t="s">
-        <v>61</v>
+        <v>144</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" s="3"/>
-      <c r="B63" s="12"/>
+      <c r="B63" s="24"/>
       <c r="C63" s="4" t="s">
-        <v>6</v>
+        <v>145</v>
       </c>
       <c r="D63" s="8" t="s">
-        <v>62</v>
+        <v>146</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" s="3"/>
-      <c r="B64" s="10" t="s">
-        <v>5</v>
-      </c>
+      <c r="B64" s="23"/>
       <c r="C64" s="4" t="s">
-        <v>4</v>
+        <v>147</v>
       </c>
       <c r="D64" s="8" t="s">
-        <v>63</v>
+        <v>148</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" s="3"/>
-      <c r="B65" s="12"/>
-      <c r="C65" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="D65" s="8" t="s">
-        <v>64</v>
+      <c r="B65" s="22" t="s">
+        <v>8</v>
+      </c>
+      <c r="C65" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D65" s="7" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" s="3"/>
-      <c r="B66" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="C66" s="4" t="s">
-        <v>133</v>
-      </c>
-      <c r="D66" s="8" t="s">
-        <v>134</v>
+      <c r="B66" s="24"/>
+      <c r="C66" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D66" s="7" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" s="3"/>
-      <c r="B67" s="11"/>
-      <c r="C67" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="D67" s="8" t="s">
-        <v>136</v>
+      <c r="B67" s="24"/>
+      <c r="C67" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D67" s="7" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" s="3"/>
-      <c r="B68" s="11"/>
-      <c r="C68" s="4" t="s">
-        <v>137</v>
-      </c>
-      <c r="D68" s="8" t="s">
-        <v>138</v>
+      <c r="B68" s="24"/>
+      <c r="C68" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D68" s="7" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" s="3"/>
-      <c r="B69" s="11"/>
-      <c r="C69" s="4" t="s">
-        <v>139</v>
-      </c>
-      <c r="D69" s="8" t="s">
-        <v>140</v>
+      <c r="B69" s="24"/>
+      <c r="C69" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D69" s="17" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" s="3"/>
-      <c r="B70" s="11"/>
-      <c r="C70" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="D70" s="8" t="s">
-        <v>142</v>
+      <c r="B70" s="23"/>
+      <c r="C70" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" s="3"/>
-      <c r="B71" s="12"/>
-      <c r="C71" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="D71" s="8" t="s">
-        <v>144</v>
+      <c r="B71" s="22" t="s">
+        <v>202</v>
+      </c>
+      <c r="C71" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="D71" s="9" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A72" s="13"/>
-      <c r="B72" s="14" t="s">
+      <c r="A72" s="3"/>
+      <c r="B72" s="23"/>
+      <c r="C72" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="D72" s="9" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A73" s="3"/>
+      <c r="B73" s="22" t="s">
+        <v>2</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="D73" s="8" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A74" s="3"/>
+      <c r="B74" s="24"/>
+      <c r="C74" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="D74" s="8" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A75" s="3"/>
+      <c r="B75" s="24"/>
+      <c r="C75" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D75" s="8" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A76" s="3"/>
+      <c r="B76" s="24"/>
+      <c r="C76" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="D76" s="8" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A77" s="3"/>
+      <c r="B77" s="24"/>
+      <c r="C77" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="D77" s="8" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A78" s="3"/>
+      <c r="B78" s="23"/>
+      <c r="C78" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="D78" s="8" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A79" s="10"/>
+      <c r="B79" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="C72" s="15" t="s">
+      <c r="C79" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="D72" s="16" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A73" s="13"/>
-      <c r="B73" s="17"/>
-      <c r="C73" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="D73" s="18" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A74" s="13"/>
-      <c r="B74" s="19"/>
-      <c r="C74" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="D74" s="18" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A75" s="20"/>
-      <c r="B75" s="21" t="s">
+      <c r="D79" s="12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A80" s="10"/>
+      <c r="B80" s="26"/>
+      <c r="C80" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D80" s="13" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A81" s="10"/>
+      <c r="B81" s="27"/>
+      <c r="C81" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D81" s="13" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A82" s="14"/>
+      <c r="B82" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="C82" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D82" s="12" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A83" s="14"/>
+      <c r="B83" s="20"/>
+      <c r="C83" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D83" s="12" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A84" s="14"/>
+      <c r="B84" s="20"/>
+      <c r="C84" s="11" t="s">
+        <v>90</v>
+      </c>
+      <c r="D84" s="18" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A85" s="14"/>
+      <c r="B85" s="20"/>
+      <c r="C85" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="D85" s="12" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A86" s="14"/>
+      <c r="B86" s="20"/>
+      <c r="C86" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="D86" s="12" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A87" s="14"/>
+      <c r="B87" s="20"/>
+      <c r="C87" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="D87" s="12" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A88" s="14"/>
+      <c r="B88" s="20"/>
+      <c r="C88" s="11" t="s">
+        <v>97</v>
+      </c>
+      <c r="D88" s="12" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A89" s="14"/>
+      <c r="B89" s="20"/>
+      <c r="C89" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="D89" s="12" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A90" s="14"/>
+      <c r="B90" s="20"/>
+      <c r="C90" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="D90" s="12" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A91" s="14"/>
+      <c r="B91" s="20"/>
+      <c r="C91" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="C75" s="15" t="s">
+      <c r="D91" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="D75" s="16" t="s">
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A92" s="14"/>
+      <c r="B92" s="20"/>
+      <c r="C92" s="11" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A76" s="20"/>
-      <c r="B76" s="22"/>
-      <c r="C76" s="15" t="s">
+      <c r="D92" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="D76" s="16" t="s">
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A93" s="14"/>
+      <c r="B93" s="20"/>
+      <c r="C93" s="11" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="77" spans="1:4" ht="27" x14ac:dyDescent="0.3">
-      <c r="A77" s="20"/>
-      <c r="B77" s="22"/>
-      <c r="C77" s="15" t="s">
+      <c r="D93" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="D77" s="27" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A78" s="20"/>
-      <c r="B78" s="22"/>
-      <c r="C78" s="15" t="s">
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A94" s="14"/>
+      <c r="B94" s="20"/>
+      <c r="C94" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="D78" s="16" t="s">
+      <c r="D94" s="12" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A79" s="20"/>
-      <c r="B79" s="22"/>
-      <c r="C79" s="15" t="s">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A95" s="14"/>
+      <c r="B95" s="20"/>
+      <c r="C95" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="D79" s="16" t="s">
+      <c r="D95" s="12" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A80" s="20"/>
-      <c r="B80" s="22"/>
-      <c r="C80" s="15" t="s">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A96" s="14"/>
+      <c r="B96" s="21"/>
+      <c r="C96" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="D80" s="16" t="s">
+      <c r="D96" s="12" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A81" s="20"/>
-      <c r="B81" s="22"/>
-      <c r="C81" s="15" t="s">
-        <v>115</v>
-      </c>
-      <c r="D81" s="16" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A82" s="20"/>
-      <c r="B82" s="22"/>
-      <c r="C82" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="D82" s="16" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A83" s="20"/>
-      <c r="B83" s="22"/>
-      <c r="C83" s="15" t="s">
-        <v>119</v>
-      </c>
-      <c r="D83" s="16" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A84" s="20"/>
-      <c r="B84" s="22"/>
-      <c r="C84" s="15" t="s">
-        <v>121</v>
-      </c>
-      <c r="D84" s="16" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A85" s="20"/>
-      <c r="B85" s="22"/>
-      <c r="C85" s="15" t="s">
-        <v>123</v>
-      </c>
-      <c r="D85" s="16" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A86" s="20"/>
-      <c r="B86" s="22"/>
-      <c r="C86" s="15" t="s">
-        <v>125</v>
-      </c>
-      <c r="D86" s="16" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A87" s="20"/>
-      <c r="B87" s="22"/>
-      <c r="C87" s="15" t="s">
-        <v>127</v>
-      </c>
-      <c r="D87" s="16" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A88" s="20"/>
-      <c r="B88" s="22"/>
-      <c r="C88" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="D88" s="16" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A89" s="20"/>
-      <c r="B89" s="23"/>
-      <c r="C89" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="D89" s="16" t="s">
-        <v>132</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="14">
-    <mergeCell ref="B75:B89"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="B4:B7"/>
-    <mergeCell ref="B8:B15"/>
-    <mergeCell ref="B16:B19"/>
-    <mergeCell ref="B22:B35"/>
-    <mergeCell ref="B36:B42"/>
-    <mergeCell ref="B66:B71"/>
-    <mergeCell ref="B43:B53"/>
-    <mergeCell ref="B54:B59"/>
-    <mergeCell ref="B60:B63"/>
-    <mergeCell ref="B64:B65"/>
-    <mergeCell ref="B72:B74"/>
+  <mergeCells count="13">
+    <mergeCell ref="B82:B96"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="B2:B14"/>
+    <mergeCell ref="B15:B18"/>
+    <mergeCell ref="B19:B26"/>
+    <mergeCell ref="B27:B30"/>
+    <mergeCell ref="B33:B46"/>
+    <mergeCell ref="B47:B53"/>
+    <mergeCell ref="B73:B78"/>
+    <mergeCell ref="B54:B64"/>
+    <mergeCell ref="B65:B70"/>
+    <mergeCell ref="B79:B81"/>
+    <mergeCell ref="B71:B72"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2201,15 +2304,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="문서" ma:contentTypeID="0x01010055643D1FCDD1AF449E52FCC5650E658B" ma:contentTypeVersion="14" ma:contentTypeDescription="새 문서를 만듭니다." ma:contentTypeScope="" ma:versionID="647bdb025269980e27106cc2d7c93b4b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e9585e3e-8dde-4558-9020-300460070f66" xmlns:ns3="fdbd0ee6-c1ce-4682-bf4d-b990274ef7f9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d9d8955b532099d955db877a9cb0cef3" ns2:_="" ns3:_="">
     <xsd:import namespace="e9585e3e-8dde-4558-9020-300460070f66"/>
@@ -2422,6 +2516,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -2434,14 +2537,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86FB0506-72B3-4F03-B05C-01BAB7410BED}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6B3FA20A-BD9F-4422-9B89-7C75BEBC07A8}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2460,6 +2555,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{86FB0506-72B3-4F03-B05C-01BAB7410BED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DDE60D44-15A8-45C5-B02F-5E97D9FCFB03}">
   <ds:schemaRefs>

</xml_diff>